<commit_message>
Add FR-31 availability referral and use team workbook
Unavailable items stay on the list with a referral to the nearest store
with stock or "ask staff"; the app now reads data/product_catalogue.xlsx
with 5 stores. Requested: implement FR-31, TC-38 without preselection.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EimuL5ZzreqsH6e3579jk7
</commit_message>
<xml_diff>
--- a/data/product_catalogue.xlsx
+++ b/data/product_catalogue.xlsx
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N74"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -580,6 +580,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -649,6 +650,31 @@
       <c r="N4" s="3" t="inlineStr">
         <is>
           <t>safety_note</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="inlineStr">
+        <is>
+          <t>variant_group</t>
+        </is>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>pack_qty</t>
+        </is>
+      </c>
+      <c r="Q4" s="3" t="inlineStr">
+        <is>
+          <t>pack_unit</t>
+        </is>
+      </c>
+      <c r="R4" s="3" t="inlineStr">
+        <is>
+          <t>specs</t>
+        </is>
+      </c>
+      <c r="S4" s="3" t="inlineStr">
+        <is>
+          <t>data_note</t>
         </is>
       </c>
     </row>
@@ -709,6 +735,20 @@
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>interior-wall-paint-matt</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -767,6 +807,20 @@
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>interior-wall-paint-matt</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -825,6 +879,20 @@
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>colour-wall-paint</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -883,6 +951,20 @@
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>colour-wall-paint</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -941,6 +1023,20 @@
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>wood-varnish</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -999,6 +1095,20 @@
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>wood-stain</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1061,6 +1171,20 @@
           <t>Use in ventilated area</t>
         </is>
       </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>metal-protection-paint</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -1115,6 +1239,20 @@
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>paint-roller-set</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -1169,6 +1307,20 @@
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>flat-brush-set</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -1227,6 +1379,20 @@
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>masking-tape</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -1285,6 +1451,20 @@
         </is>
       </c>
       <c r="N15" s="5" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>drop-cloth</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -1343,6 +1523,20 @@
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>wall-filler</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1397,6 +1591,20 @@
         </is>
       </c>
       <c r="N17" s="5" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>sanding-paper-set</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -1451,6 +1659,20 @@
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>led-bulb-e27</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1505,6 +1727,20 @@
         </is>
       </c>
       <c r="N19" s="5" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>led-bulb-gu10</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1563,6 +1799,20 @@
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>extension-cord-3-way</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1625,6 +1875,20 @@
           <t>Electrical work only by a qualified electrician</t>
         </is>
       </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>installation-cable-nym-j</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
@@ -1683,6 +1947,20 @@
           <t>Does not replace professional measurement</t>
         </is>
       </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>voltage-tester</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1745,6 +2023,20 @@
           <t>Electrical work only by a qualified electrician</t>
         </is>
       </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>light-switch-flush-mounted</t>
+        </is>
+      </c>
+      <c r="P23" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1799,6 +2091,20 @@
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>tap-washer-set</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1857,6 +2163,20 @@
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr"/>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>ptfe-thread-seal-tape</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1915,6 +2235,20 @@
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr"/>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>shower-hose</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1973,6 +2307,20 @@
         </is>
       </c>
       <c r="N27" s="5" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>sink-siphon</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
@@ -2031,6 +2379,20 @@
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>pipe-wrench</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -2085,6 +2447,20 @@
         </is>
       </c>
       <c r="N29" s="5" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>garden-hose</t>
+        </is>
+      </c>
+      <c r="P29" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
@@ -2135,6 +2511,20 @@
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>potting-soil</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -2189,6 +2579,20 @@
         </is>
       </c>
       <c r="N31" s="5" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>work-gloves</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
@@ -2247,6 +2651,20 @@
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr"/>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>safety-goggles</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -2305,6 +2723,20 @@
         </is>
       </c>
       <c r="N33" s="5" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>dust-mask-ffp2</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
@@ -2359,6 +2791,20 @@
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr"/>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>claw-hammer</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2413,6 +2859,20 @@
         </is>
       </c>
       <c r="N35" s="5" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>screwdriver-set</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2471,6 +2931,20 @@
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>spirit-level</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2521,6 +2995,20 @@
         </is>
       </c>
       <c r="N37" s="5" t="inlineStr"/>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>tape-measure</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2579,6 +3067,20 @@
           <t>Always scan wall before drilling</t>
         </is>
       </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>stud-and-cable-detector</t>
+        </is>
+      </c>
+      <c r="P38" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2637,6 +3139,24 @@
         </is>
       </c>
       <c r="N39" s="5" t="inlineStr"/>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>masonry-drill-bit</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>diameter_mm=6</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2695,6 +3215,24 @@
         </is>
       </c>
       <c r="N40" s="5" t="inlineStr"/>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>masonry-drill-bit</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>diameter_mm=8</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2753,6 +3291,24 @@
         </is>
       </c>
       <c r="N41" s="5" t="inlineStr"/>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>masonry-drill-bit</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>diameter_mm=10</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2807,6 +3363,20 @@
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr"/>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>wood-drill-bit-set</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2865,6 +3435,20 @@
         </is>
       </c>
       <c r="N43" s="5" t="inlineStr"/>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>cordless-drill-driver</t>
+        </is>
+      </c>
+      <c r="P43" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2927,6 +3511,20 @@
           <t>Wear safety goggles</t>
         </is>
       </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>hammer-drill</t>
+        </is>
+      </c>
+      <c r="P44" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2989,6 +3587,20 @@
           <t>Wear safety goggles</t>
         </is>
       </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>jigsaw</t>
+        </is>
+      </c>
+      <c r="P45" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -3051,6 +3663,20 @@
           <t>Wear dust mask</t>
         </is>
       </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>orbital-sander</t>
+        </is>
+      </c>
+      <c r="P46" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3115,6 +3741,24 @@
         </is>
       </c>
       <c r="N47" s="5" t="inlineStr"/>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>universal-wall-plug</t>
+        </is>
+      </c>
+      <c r="P47" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>diameter_mm=6</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3179,6 +3823,24 @@
         </is>
       </c>
       <c r="N48" s="5" t="inlineStr"/>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>universal-wall-plug</t>
+        </is>
+      </c>
+      <c r="P48" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>diameter_mm=8</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -3243,6 +3905,24 @@
         </is>
       </c>
       <c r="N49" s="5" t="inlineStr"/>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>heavy-duty-wall-plug</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>diameter_mm=10</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
@@ -3307,6 +3987,24 @@
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr"/>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>plasterboard-anchor</t>
+        </is>
+      </c>
+      <c r="P50" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
+        <is>
+          <t>thread=M5</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
@@ -3375,6 +4073,24 @@
           <t>Over 50 kg: consider a professional</t>
         </is>
       </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>heavy-duty-anchor-bolt</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>thread=M8;length_mm=80</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
@@ -3435,6 +4151,24 @@
         </is>
       </c>
       <c r="N52" s="5" t="inlineStr"/>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>wood-screw</t>
+        </is>
+      </c>
+      <c r="P52" t="n">
+        <v>100</v>
+      </c>
+      <c r="Q52" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R52" t="inlineStr">
+        <is>
+          <t>diameter_mm=4;length_mm=40</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
@@ -3495,6 +4229,24 @@
         </is>
       </c>
       <c r="N53" s="5" t="inlineStr"/>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>wood-screw</t>
+        </is>
+      </c>
+      <c r="P53" t="n">
+        <v>50</v>
+      </c>
+      <c r="Q53" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R53" t="inlineStr">
+        <is>
+          <t>diameter_mm=5;length_mm=50</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
@@ -3555,6 +4307,24 @@
         </is>
       </c>
       <c r="N54" s="5" t="inlineStr"/>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>wood-screw</t>
+        </is>
+      </c>
+      <c r="P54" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q54" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R54" t="inlineStr">
+        <is>
+          <t>diameter_mm=6;length_mm=60</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
@@ -3598,7 +4368,11 @@
       <c r="I55" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="J55" s="5" t="inlineStr"/>
+      <c r="J55" s="5" t="inlineStr">
+        <is>
+          <t>brick;plasterboard</t>
+        </is>
+      </c>
       <c r="K55" s="5" t="inlineStr">
         <is>
           <t>P030</t>
@@ -3615,6 +4389,25 @@
         </is>
       </c>
       <c r="N55" s="5" t="inlineStr"/>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>picture-hook-set</t>
+        </is>
+      </c>
+      <c r="P55" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q55" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R55" t="inlineStr"/>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>suitable_wall_types added for the app – team to verify (SR-10)</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
@@ -3679,6 +4472,20 @@
         </is>
       </c>
       <c r="N56" s="5" t="inlineStr"/>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>mounting-adhesive</t>
+        </is>
+      </c>
+      <c r="P56" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q56" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
@@ -3733,6 +4540,20 @@
         </is>
       </c>
       <c r="N57" s="5" t="inlineStr"/>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>wood-glue</t>
+        </is>
+      </c>
+      <c r="P57" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q57" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
@@ -3791,6 +4612,20 @@
         </is>
       </c>
       <c r="N58" s="5" t="inlineStr"/>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>sanitary-silicone</t>
+        </is>
+      </c>
+      <c r="P58" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q58" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
@@ -3849,6 +4684,20 @@
         </is>
       </c>
       <c r="N59" s="5" t="inlineStr"/>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>sanitary-silicone</t>
+        </is>
+      </c>
+      <c r="P59" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
@@ -3907,6 +4756,20 @@
         </is>
       </c>
       <c r="N60" s="5" t="inlineStr"/>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>acrylic-sealant</t>
+        </is>
+      </c>
+      <c r="P60" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -3961,6 +4824,20 @@
         </is>
       </c>
       <c r="N61" s="5" t="inlineStr"/>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>caulking-gun</t>
+        </is>
+      </c>
+      <c r="P61" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q61" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
@@ -4021,6 +4898,24 @@
         </is>
       </c>
       <c r="N62" s="5" t="inlineStr"/>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>shelf-bracket</t>
+        </is>
+      </c>
+      <c r="P62" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q62" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R62" t="inlineStr">
+        <is>
+          <t>arm_mm=150</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -4081,6 +4976,24 @@
         </is>
       </c>
       <c r="N63" s="5" t="inlineStr"/>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>shelf-bracket</t>
+        </is>
+      </c>
+      <c r="P63" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>arm_mm=200</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -4141,6 +5054,24 @@
         </is>
       </c>
       <c r="N64" s="5" t="inlineStr"/>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>shelf-bracket-heavy-duty</t>
+        </is>
+      </c>
+      <c r="P64" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q64" t="inlineStr">
+        <is>
+          <t>pcs</t>
+        </is>
+      </c>
+      <c r="R64" t="inlineStr">
+        <is>
+          <t>arm_mm=250</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
@@ -4201,6 +5132,20 @@
         </is>
       </c>
       <c r="N65" s="5" t="inlineStr"/>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>floating-shelf-kit</t>
+        </is>
+      </c>
+      <c r="P65" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
@@ -4261,6 +5206,20 @@
         </is>
       </c>
       <c r="N66" s="5" t="inlineStr"/>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>wall-rail-system</t>
+        </is>
+      </c>
+      <c r="P66" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q66" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -4321,6 +5280,24 @@
         </is>
       </c>
       <c r="N67" s="5" t="inlineStr"/>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>shelf-board</t>
+        </is>
+      </c>
+      <c r="P67" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R67" t="inlineStr">
+        <is>
+          <t>length_mm=800;depth_mm=200;thickness_mm=18</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -4381,6 +5358,24 @@
         </is>
       </c>
       <c r="N68" s="5" t="inlineStr"/>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>shelf-board</t>
+        </is>
+      </c>
+      <c r="P68" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q68" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R68" t="inlineStr">
+        <is>
+          <t>length_mm=800;depth_mm=250;thickness_mm=18</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -4439,6 +5434,20 @@
         </is>
       </c>
       <c r="N69" s="5" t="inlineStr"/>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>wooden-block</t>
+        </is>
+      </c>
+      <c r="P69" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q69" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4497,6 +5506,20 @@
         </is>
       </c>
       <c r="N70" s="5" t="inlineStr"/>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>wooden-block</t>
+        </is>
+      </c>
+      <c r="P70" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q70" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
@@ -4555,6 +5578,20 @@
         </is>
       </c>
       <c r="N71" s="5" t="inlineStr"/>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>batten</t>
+        </is>
+      </c>
+      <c r="P71" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q71" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
@@ -4613,6 +5650,20 @@
         </is>
       </c>
       <c r="N72" s="5" t="inlineStr"/>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>square-timber</t>
+        </is>
+      </c>
+      <c r="P72" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q72" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
@@ -4671,6 +5722,20 @@
         </is>
       </c>
       <c r="N73" s="5" t="inlineStr"/>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>glued-laminated-panel</t>
+        </is>
+      </c>
+      <c r="P73" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
@@ -4729,6 +5794,20 @@
         </is>
       </c>
       <c r="N74" s="5" t="inlineStr"/>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>mdf-board</t>
+        </is>
+      </c>
+      <c r="P74" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q74" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="R74" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:N74"/>

</xml_diff>

<commit_message>
Add 120 cm shelf board P103 to the product catalogue
Shelves of 81-120 cm (25 cm deep) were impossible with 80 cm boards only.
Sample price, load rating and stock. Prompt: add a 120 cm shelf board with a
load rating.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013GEFV7GrcoHwDr8wsfQpUb
</commit_message>
<xml_diff>
--- a/data/product_catalogue.xlsx
+++ b/data/product_catalogue.xlsx
@@ -812,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U106"/>
+  <dimension ref="A1:U107"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="34" min="1" max="1"/>
@@ -9747,6 +9747,103 @@
       <c r="U106" s="46" t="inlineStr">
         <is>
           <t>new 27 Oct 2026 – generic sample product</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>P103</t>
+        </is>
+      </c>
+      <c r="B107" s="46" t="inlineStr">
+        <is>
+          <t>Shelf board</t>
+        </is>
+      </c>
+      <c r="C107" s="46" t="inlineStr">
+        <is>
+          <t>Regalboden</t>
+        </is>
+      </c>
+      <c r="D107" s="46" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="E107" s="46" t="inlineStr">
+        <is>
+          <t>Regalsysteme</t>
+        </is>
+      </c>
+      <c r="F107" s="46" t="inlineStr">
+        <is>
+          <t>1200 x 250 x 18 mm</t>
+        </is>
+      </c>
+      <c r="G107" s="46" t="inlineStr">
+        <is>
+          <t>Melamine-coated shelf board, can be cut to length</t>
+        </is>
+      </c>
+      <c r="H107" s="46" t="inlineStr">
+        <is>
+          <t>Chipboard</t>
+        </is>
+      </c>
+      <c r="I107" s="46" t="inlineStr">
+        <is>
+          <t>Oak decor</t>
+        </is>
+      </c>
+      <c r="J107" s="47" t="n">
+        <v>19.99</v>
+      </c>
+      <c r="K107" s="46" t="n">
+        <v>25</v>
+      </c>
+      <c r="L107" s="46" t="n"/>
+      <c r="M107" s="46" t="inlineStr">
+        <is>
+          <t>P059;P060;P041</t>
+        </is>
+      </c>
+      <c r="N107" s="46" t="inlineStr">
+        <is>
+          <t>shelf hanging</t>
+        </is>
+      </c>
+      <c r="O107" s="46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P107" s="46" t="inlineStr">
+        <is>
+          <t>Use 3 brackets, max. 60 cm apart. Rated load applies to the whole board.</t>
+        </is>
+      </c>
+      <c r="Q107" s="46" t="inlineStr">
+        <is>
+          <t>shelf-board</t>
+        </is>
+      </c>
+      <c r="R107" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S107" s="46" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="T107" s="46" t="inlineStr">
+        <is>
+          <t>length_mm=1200;depth_mm=250;thickness_mm=18</t>
+        </is>
+      </c>
+      <c r="U107" s="46" t="inlineStr">
+        <is>
+          <t>added 27 Oct 2026 on request – generic sample product; price and load rating are sample values (team to verify)</t>
         </is>
       </c>
     </row>
@@ -18292,6 +18389,88 @@
       </c>
       <c r="V106" s="55" t="n">
         <v>6</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="45" t="inlineStr">
+        <is>
+          <t>P103</t>
+        </is>
+      </c>
+      <c r="B107" s="46" t="inlineStr">
+        <is>
+          <t>Shelf board</t>
+        </is>
+      </c>
+      <c r="C107" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D107" s="44" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="E107" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F107" s="44" t="n">
+        <v>9</v>
+      </c>
+      <c r="G107" s="46" t="n">
+        <v>4</v>
+      </c>
+      <c r="H107" s="46" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="I107" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="J107" s="46" t="n">
+        <v>12</v>
+      </c>
+      <c r="K107" s="53" t="n">
+        <v>15</v>
+      </c>
+      <c r="L107" s="53" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="M107" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="N107" s="53" t="n">
+        <v>7</v>
+      </c>
+      <c r="O107" s="54" t="n">
+        <v>15</v>
+      </c>
+      <c r="P107" s="54" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="Q107" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="R107" s="54" t="n">
+        <v>10</v>
+      </c>
+      <c r="S107" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="T107" s="55" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="U107" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="V107" s="55" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="35">

</xml_diff>

<commit_message>
Add 120 cm shelf board P104 with 20 cm depth
20 cm deep shelves above 80 cm still stopped. Sample price, rating and stock;
size-message test now uses a catalogue copy without P104.
Prompt: also add a 120 cm board with 20 cm depth.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013GEFV7GrcoHwDr8wsfQpUb
</commit_message>
<xml_diff>
--- a/data/product_catalogue.xlsx
+++ b/data/product_catalogue.xlsx
@@ -812,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U107"/>
+  <dimension ref="A1:U108"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="34" min="1" max="1"/>
@@ -9847,6 +9847,103 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="45" t="inlineStr">
+        <is>
+          <t>P104</t>
+        </is>
+      </c>
+      <c r="B108" s="46" t="inlineStr">
+        <is>
+          <t>Shelf board</t>
+        </is>
+      </c>
+      <c r="C108" s="46" t="inlineStr">
+        <is>
+          <t>Regalboden</t>
+        </is>
+      </c>
+      <c r="D108" s="46" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="E108" s="46" t="inlineStr">
+        <is>
+          <t>Regalsysteme</t>
+        </is>
+      </c>
+      <c r="F108" s="46" t="inlineStr">
+        <is>
+          <t>1200 x 200 x 18 mm</t>
+        </is>
+      </c>
+      <c r="G108" s="46" t="inlineStr">
+        <is>
+          <t>Melamine-coated shelf board, can be cut to length</t>
+        </is>
+      </c>
+      <c r="H108" s="46" t="inlineStr">
+        <is>
+          <t>Chipboard</t>
+        </is>
+      </c>
+      <c r="I108" s="46" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="J108" s="47" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="K108" s="46" t="n">
+        <v>20</v>
+      </c>
+      <c r="L108" s="46" t="n"/>
+      <c r="M108" s="46" t="inlineStr">
+        <is>
+          <t>P058;P059;P041</t>
+        </is>
+      </c>
+      <c r="N108" s="46" t="inlineStr">
+        <is>
+          <t>shelf hanging</t>
+        </is>
+      </c>
+      <c r="O108" s="46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P108" s="46" t="inlineStr">
+        <is>
+          <t>Use 3 brackets, max. 60 cm apart. Rated load applies to the whole board.</t>
+        </is>
+      </c>
+      <c r="Q108" s="46" t="inlineStr">
+        <is>
+          <t>shelf-board</t>
+        </is>
+      </c>
+      <c r="R108" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S108" s="46" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="T108" s="46" t="inlineStr">
+        <is>
+          <t>length_mm=1200;depth_mm=200;thickness_mm=18</t>
+        </is>
+      </c>
+      <c r="U108" s="46" t="inlineStr">
+        <is>
+          <t>added 27 Oct 2026 on request – generic sample product; price and load rating are sample values (team to verify)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:U106"/>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
@@ -9861,7 +9958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V113"/>
+  <dimension ref="A1:V114"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="34" min="1" max="1"/>
@@ -18474,44 +18571,126 @@
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="35">
-      <c r="A108" s="38" t="inlineStr">
+      <c r="A108" s="45" t="inlineStr">
+        <is>
+          <t>P104</t>
+        </is>
+      </c>
+      <c r="B108" s="46" t="inlineStr">
+        <is>
+          <t>Shelf board</t>
+        </is>
+      </c>
+      <c r="C108" s="44" t="n">
+        <v>8</v>
+      </c>
+      <c r="D108" s="44" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="E108" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F108" s="44" t="n">
+        <v>11</v>
+      </c>
+      <c r="G108" s="46" t="n">
+        <v>4</v>
+      </c>
+      <c r="H108" s="46" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="I108" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="J108" s="46" t="n">
+        <v>8</v>
+      </c>
+      <c r="K108" s="53" t="n">
+        <v>15</v>
+      </c>
+      <c r="L108" s="53" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="M108" s="53" t="n">
+        <v>3</v>
+      </c>
+      <c r="N108" s="53" t="n">
+        <v>9</v>
+      </c>
+      <c r="O108" s="54" t="n">
+        <v>15</v>
+      </c>
+      <c r="P108" s="54" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="Q108" s="54" t="n">
+        <v>3</v>
+      </c>
+      <c r="R108" s="54" t="n">
+        <v>12</v>
+      </c>
+      <c r="S108" s="55" t="n">
+        <v>4</v>
+      </c>
+      <c r="T108" s="55" t="inlineStr">
+        <is>
+          <t>Shelving</t>
+        </is>
+      </c>
+      <c r="U108" s="55" t="n">
+        <v>3</v>
+      </c>
+      <c r="V108" s="55" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="109" ht="15" customHeight="1" s="35">
+      <c r="A109" s="38" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="109" ht="15" customHeight="1" s="35">
-      <c r="A109" s="58" t="n"/>
-      <c r="B109" s="59" t="inlineStr">
+    <row r="110" ht="15" customHeight="1" s="35">
+      <c r="A110" s="58" t="n"/>
+      <c r="B110" s="59" t="inlineStr">
         <is>
           <t>qty 0 = out of stock (app refers to nearest store with stock, FR-31)</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="15" customHeight="1" s="35">
-      <c r="A110" s="60" t="n"/>
-      <c r="B110" s="59" t="inlineStr">
+    <row r="111" ht="15" customHeight="1" s="35">
+      <c r="A111" s="60" t="n"/>
+      <c r="B111" s="59" t="inlineStr">
         <is>
           <t>empty = not carried in this store (FR-31)</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="15" customHeight="1" s="35">
-      <c r="B111" s="59" t="inlineStr">
-        <is>
-          <t>Demo cases: P044 out of stock in ERL-OST · P059 not carried in NUE-REG · P064 out of stock in NUE-BAY</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="35">
       <c r="B112" s="59" t="inlineStr">
         <is>
-          <t>ERL-OST uses the original catalogue layout; other stores: same aisle names, different aisle numbers and stock (generated sample data). P071–P102: generated sample stock, all in stock.</t>
+          <t>Demo cases: P044 out of stock in ERL-OST · P059 not carried in NUE-REG · P064 out of stock in NUE-BAY</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="35">
       <c r="B113" s="59" t="inlineStr">
+        <is>
+          <t>ERL-OST uses the original catalogue layout; other stores: same aisle names, different aisle numbers and stock (generated sample data). P071–P102: generated sample stock, all in stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="59" t="inlineStr">
         <is>
           <t>German aisle names: see sheet "Translations".</t>
         </is>

</xml_diff>

<commit_message>
Check sliding door sizes with overlap, height and free wall
Leaf must overlap the opening, fit the free wall and the height is now checked;
second sample leaf P105; size stops show needed vs. available in cm.
Prompt: dimensions make little sense – implement it with a second door leaf.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013GEFV7GrcoHwDr8wsfQpUb
</commit_message>
<xml_diff>
--- a/data/product_catalogue.xlsx
+++ b/data/product_catalogue.xlsx
@@ -812,7 +812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:U108"/>
+  <dimension ref="A1:U109"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="34" min="1" max="1"/>
@@ -9288,12 +9288,12 @@
       </c>
       <c r="T101" s="46" t="inlineStr">
         <is>
-          <t>width_mm=900;weight_kg=25</t>
+          <t>width_mm=900;weight_kg=25;height_mm=2035</t>
         </is>
       </c>
       <c r="U101" s="46" t="inlineStr">
         <is>
-          <t>new 27 Oct 2026 – generic sample product</t>
+          <t>new 27 Oct 2026 – generic sample product; specs height_mm=2035 added for the app from the size</t>
         </is>
       </c>
     </row>
@@ -9941,6 +9941,101 @@
       <c r="U108" s="46" t="inlineStr">
         <is>
           <t>added 27 Oct 2026 on request – generic sample product; price and load rating are sample values (team to verify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="45" t="inlineStr">
+        <is>
+          <t>P105</t>
+        </is>
+      </c>
+      <c r="B109" s="46" t="inlineStr">
+        <is>
+          <t>Wooden sliding door leaf</t>
+        </is>
+      </c>
+      <c r="C109" s="46" t="inlineStr">
+        <is>
+          <t>Holz-Schiebetürblatt</t>
+        </is>
+      </c>
+      <c r="D109" s="46" t="inlineStr">
+        <is>
+          <t>Sliding doors</t>
+        </is>
+      </c>
+      <c r="E109" s="46" t="inlineStr">
+        <is>
+          <t>Schiebetüren</t>
+        </is>
+      </c>
+      <c r="F109" s="46" t="inlineStr">
+        <is>
+          <t>1000 x 2135 mm</t>
+        </is>
+      </c>
+      <c r="G109" s="46" t="inlineStr">
+        <is>
+          <t>Wide door leaf for wall-mounted sliding door systems</t>
+        </is>
+      </c>
+      <c r="H109" s="46" t="inlineStr">
+        <is>
+          <t>Wood composite</t>
+        </is>
+      </c>
+      <c r="I109" s="46" t="inlineStr">
+        <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="J109" s="47" t="n">
+        <v>179</v>
+      </c>
+      <c r="K109" s="46" t="n"/>
+      <c r="L109" s="46" t="n"/>
+      <c r="M109" s="46" t="inlineStr">
+        <is>
+          <t>P096;P099</t>
+        </is>
+      </c>
+      <c r="N109" s="46" t="inlineStr">
+        <is>
+          <t>installing a sliding door</t>
+        </is>
+      </c>
+      <c r="O109" s="46" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="P109" s="46" t="inlineStr">
+        <is>
+          <t>Carry with two people.</t>
+        </is>
+      </c>
+      <c r="Q109" s="46" t="inlineStr">
+        <is>
+          <t>wooden-sliding-door-leaf</t>
+        </is>
+      </c>
+      <c r="R109" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="S109" s="46" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="T109" s="46" t="inlineStr">
+        <is>
+          <t>width_mm=1000;height_mm=2135;weight_kg=30</t>
+        </is>
+      </c>
+      <c r="U109" s="46" t="inlineStr">
+        <is>
+          <t>added 27 Oct 2026 on request – generic sample product; price and weight are sample values (team to verify)</t>
         </is>
       </c>
     </row>
@@ -9958,7 +10053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V114"/>
+  <dimension ref="A1:V115"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="10" customWidth="1" style="34" min="1" max="1"/>
@@ -18653,44 +18748,126 @@
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="35">
-      <c r="A109" s="38" t="inlineStr">
+      <c r="A109" s="45" t="inlineStr">
+        <is>
+          <t>P105</t>
+        </is>
+      </c>
+      <c r="B109" s="46" t="inlineStr">
+        <is>
+          <t>Wooden sliding door leaf</t>
+        </is>
+      </c>
+      <c r="C109" s="44" t="n">
+        <v>10</v>
+      </c>
+      <c r="D109" s="44" t="inlineStr">
+        <is>
+          <t>Doors &amp; locks</t>
+        </is>
+      </c>
+      <c r="E109" s="44" t="n">
+        <v>3</v>
+      </c>
+      <c r="F109" s="44" t="n">
+        <v>4</v>
+      </c>
+      <c r="G109" s="46" t="n">
+        <v>10</v>
+      </c>
+      <c r="H109" s="46" t="inlineStr">
+        <is>
+          <t>Doors &amp; locks</t>
+        </is>
+      </c>
+      <c r="I109" s="46" t="n">
+        <v>1</v>
+      </c>
+      <c r="J109" s="46" t="n">
+        <v>3</v>
+      </c>
+      <c r="K109" s="53" t="n">
+        <v>10</v>
+      </c>
+      <c r="L109" s="53" t="inlineStr">
+        <is>
+          <t>Doors &amp; locks</t>
+        </is>
+      </c>
+      <c r="M109" s="53" t="n">
+        <v>4</v>
+      </c>
+      <c r="N109" s="53" t="n">
+        <v>5</v>
+      </c>
+      <c r="O109" s="54" t="n">
+        <v>10</v>
+      </c>
+      <c r="P109" s="54" t="inlineStr">
+        <is>
+          <t>Doors &amp; locks</t>
+        </is>
+      </c>
+      <c r="Q109" s="54" t="n">
+        <v>4</v>
+      </c>
+      <c r="R109" s="54" t="n">
+        <v>2</v>
+      </c>
+      <c r="S109" s="55" t="n">
+        <v>10</v>
+      </c>
+      <c r="T109" s="55" t="inlineStr">
+        <is>
+          <t>Doors &amp; locks</t>
+        </is>
+      </c>
+      <c r="U109" s="55" t="n">
+        <v>1</v>
+      </c>
+      <c r="V109" s="55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="110" ht="15" customHeight="1" s="35">
+      <c r="A110" s="38" t="inlineStr">
         <is>
           <t>Legend</t>
         </is>
       </c>
     </row>
-    <row r="110" ht="15" customHeight="1" s="35">
-      <c r="A110" s="58" t="n"/>
-      <c r="B110" s="59" t="inlineStr">
+    <row r="111" ht="15" customHeight="1" s="35">
+      <c r="A111" s="58" t="n"/>
+      <c r="B111" s="59" t="inlineStr">
         <is>
           <t>qty 0 = out of stock (app refers to nearest store with stock, FR-31)</t>
         </is>
       </c>
     </row>
-    <row r="111" ht="15" customHeight="1" s="35">
-      <c r="A111" s="60" t="n"/>
-      <c r="B111" s="59" t="inlineStr">
+    <row r="112" ht="15" customHeight="1" s="35">
+      <c r="A112" s="60" t="n"/>
+      <c r="B112" s="59" t="inlineStr">
         <is>
           <t>empty = not carried in this store (FR-31)</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="15" customHeight="1" s="35">
-      <c r="B112" s="59" t="inlineStr">
-        <is>
-          <t>Demo cases: P044 out of stock in ERL-OST · P059 not carried in NUE-REG · P064 out of stock in NUE-BAY</t>
         </is>
       </c>
     </row>
     <row r="113" ht="15" customHeight="1" s="35">
       <c r="B113" s="59" t="inlineStr">
         <is>
-          <t>ERL-OST uses the original catalogue layout; other stores: same aisle names, different aisle numbers and stock (generated sample data). P071–P102: generated sample stock, all in stock.</t>
+          <t>Demo cases: P044 out of stock in ERL-OST · P059 not carried in NUE-REG · P064 out of stock in NUE-BAY</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" s="59" t="inlineStr">
+        <is>
+          <t>ERL-OST uses the original catalogue layout; other stores: same aisle names, different aisle numbers and stock (generated sample data). P071–P102: generated sample stock, all in stock.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="59" t="inlineStr">
         <is>
           <t>German aisle names: see sheet "Translations".</t>
         </is>

</xml_diff>